<commit_message>
Relais Schema - Symbol und Footprint hochgeladen.
</commit_message>
<xml_diff>
--- a/Bauhalle_Zeitplan_woechentlich.xlsx
+++ b/Bauhalle_Zeitplan_woechentlich.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hueppim\Documents\Github\BauhallenUhr_New\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hueppim\Documents\Github\BauhallenUhr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C84DB9-EB8B-4805-B71B-0E699A4A7DB5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F10DA9-8EC2-45B0-99CC-8F1CA9DC77D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44385" yWindow="3855" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="79">
   <si>
     <t>Bauhalle Zeitplan wöchentlich</t>
   </si>
@@ -256,6 +256,15 @@
   </si>
   <si>
     <t>In Ordnung. Da ich mal zu viel mal zu wenig Zeit eingeschätzt hatte.</t>
+  </si>
+  <si>
+    <t>Ich habe viele Änderungen während dem Schema Zeichnen gemacht, diese Zeit hatte ich nicht auf dem Schirm.</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Dazu habe ich vergessen, die Bauteilauswahl bei Elektronische Bauteile einzuschreiben.</t>
   </si>
 </sst>
 </file>
@@ -604,7 +613,7 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -669,11 +678,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="2" xfId="10" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="4" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
@@ -682,11 +693,9 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="4" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -703,12 +712,18 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" xfId="8" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="2" xfId="10" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Excel Built-in 20% - Accent1" xfId="7" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
@@ -988,11 +1003,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="21" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="3" spans="1:19" ht="15">
       <c r="A3" s="3" t="s">
@@ -1136,194 +1151,194 @@
       </c>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="42" t="s">
+      <c r="B6" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="43" t="s">
+      <c r="E6" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="43" t="s">
+      <c r="F6" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="44" t="s">
+      <c r="G6" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="43" t="s">
+      <c r="H6" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="43" t="s">
+      <c r="I6" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="43" t="s">
+      <c r="J6" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="41"/>
-      <c r="L6" s="41"/>
-      <c r="M6" s="41"/>
-      <c r="N6" s="41"/>
-      <c r="O6" s="41"/>
-      <c r="P6" s="41"/>
-      <c r="Q6" s="41"/>
-      <c r="R6" s="41"/>
-      <c r="S6" s="45" t="s">
+      <c r="K6" s="43"/>
+      <c r="L6" s="43"/>
+      <c r="M6" s="43"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="43"/>
+      <c r="P6" s="43"/>
+      <c r="Q6" s="43"/>
+      <c r="R6" s="43"/>
+      <c r="S6" s="44" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:19">
-      <c r="A7" s="41"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="41"/>
-      <c r="J7" s="41"/>
-      <c r="K7" s="41"/>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="41"/>
-      <c r="P7" s="41"/>
-      <c r="Q7" s="41"/>
-      <c r="R7" s="41"/>
-      <c r="S7" s="45"/>
+      <c r="A7" s="43"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="43"/>
+      <c r="L7" s="43"/>
+      <c r="M7" s="43"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="43"/>
+      <c r="P7" s="43"/>
+      <c r="Q7" s="43"/>
+      <c r="R7" s="43"/>
+      <c r="S7" s="44"/>
     </row>
     <row r="8" spans="1:19">
-      <c r="A8" s="41"/>
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="41"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="41"/>
-      <c r="L8" s="41"/>
-      <c r="M8" s="41"/>
-      <c r="N8" s="41"/>
-      <c r="O8" s="41"/>
-      <c r="P8" s="41"/>
-      <c r="Q8" s="41"/>
-      <c r="R8" s="41"/>
-      <c r="S8" s="45"/>
+      <c r="A8" s="43"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="43"/>
+      <c r="N8" s="43"/>
+      <c r="O8" s="43"/>
+      <c r="P8" s="43"/>
+      <c r="Q8" s="43"/>
+      <c r="R8" s="43"/>
+      <c r="S8" s="44"/>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="41"/>
-      <c r="B9" s="41"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="41"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="41"/>
-      <c r="G9" s="41"/>
-      <c r="H9" s="41"/>
-      <c r="I9" s="41"/>
-      <c r="J9" s="41"/>
-      <c r="K9" s="41"/>
-      <c r="L9" s="41"/>
-      <c r="M9" s="41"/>
-      <c r="N9" s="41"/>
-      <c r="O9" s="41"/>
-      <c r="P9" s="41"/>
-      <c r="Q9" s="41"/>
-      <c r="R9" s="41"/>
-      <c r="S9" s="45"/>
+      <c r="A9" s="43"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="43"/>
+      <c r="K9" s="43"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="43"/>
+      <c r="N9" s="43"/>
+      <c r="O9" s="43"/>
+      <c r="P9" s="43"/>
+      <c r="Q9" s="43"/>
+      <c r="R9" s="43"/>
+      <c r="S9" s="44"/>
     </row>
     <row r="10" spans="1:19">
-      <c r="A10" s="41"/>
-      <c r="B10" s="41"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-      <c r="J10" s="41"/>
-      <c r="K10" s="41"/>
-      <c r="L10" s="41"/>
-      <c r="M10" s="41"/>
-      <c r="N10" s="41"/>
-      <c r="O10" s="41"/>
-      <c r="P10" s="41"/>
-      <c r="Q10" s="41"/>
-      <c r="R10" s="41"/>
-      <c r="S10" s="45"/>
+      <c r="A10" s="43"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="43"/>
+      <c r="I10" s="43"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="43"/>
+      <c r="L10" s="43"/>
+      <c r="M10" s="43"/>
+      <c r="N10" s="43"/>
+      <c r="O10" s="43"/>
+      <c r="P10" s="43"/>
+      <c r="Q10" s="43"/>
+      <c r="R10" s="43"/>
+      <c r="S10" s="44"/>
     </row>
     <row r="11" spans="1:19">
-      <c r="A11" s="41"/>
-      <c r="B11" s="41"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="41"/>
-      <c r="K11" s="41"/>
-      <c r="L11" s="41"/>
-      <c r="M11" s="41"/>
-      <c r="N11" s="41"/>
-      <c r="O11" s="41"/>
-      <c r="P11" s="41"/>
-      <c r="Q11" s="41"/>
-      <c r="R11" s="41"/>
-      <c r="S11" s="45"/>
+      <c r="A11" s="43"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="43"/>
+      <c r="L11" s="43"/>
+      <c r="M11" s="43"/>
+      <c r="N11" s="43"/>
+      <c r="O11" s="43"/>
+      <c r="P11" s="43"/>
+      <c r="Q11" s="43"/>
+      <c r="R11" s="43"/>
+      <c r="S11" s="44"/>
     </row>
     <row r="12" spans="1:19">
-      <c r="A12" s="41"/>
-      <c r="B12" s="41"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="41"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="41"/>
-      <c r="K12" s="41"/>
-      <c r="L12" s="41"/>
-      <c r="M12" s="41"/>
-      <c r="N12" s="41"/>
-      <c r="O12" s="41"/>
-      <c r="P12" s="41"/>
-      <c r="Q12" s="41"/>
-      <c r="R12" s="41"/>
-      <c r="S12" s="45"/>
+      <c r="A12" s="43"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="43"/>
+      <c r="I12" s="43"/>
+      <c r="J12" s="43"/>
+      <c r="K12" s="43"/>
+      <c r="L12" s="43"/>
+      <c r="M12" s="43"/>
+      <c r="N12" s="43"/>
+      <c r="O12" s="43"/>
+      <c r="P12" s="43"/>
+      <c r="Q12" s="43"/>
+      <c r="R12" s="43"/>
+      <c r="S12" s="44"/>
     </row>
     <row r="13" spans="1:19">
-      <c r="A13" s="41"/>
-      <c r="B13" s="41"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="41"/>
-      <c r="I13" s="41"/>
-      <c r="J13" s="41"/>
-      <c r="K13" s="41"/>
-      <c r="L13" s="41"/>
-      <c r="M13" s="41"/>
-      <c r="N13" s="41"/>
-      <c r="O13" s="41"/>
-      <c r="P13" s="41"/>
-      <c r="Q13" s="41"/>
-      <c r="R13" s="41"/>
-      <c r="S13" s="45"/>
+      <c r="A13" s="43"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="43"/>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43"/>
+      <c r="K13" s="43"/>
+      <c r="L13" s="43"/>
+      <c r="M13" s="43"/>
+      <c r="N13" s="43"/>
+      <c r="O13" s="43"/>
+      <c r="P13" s="43"/>
+      <c r="Q13" s="43"/>
+      <c r="R13" s="43"/>
+      <c r="S13" s="44"/>
     </row>
     <row r="14" spans="1:19" ht="30" customHeight="1">
       <c r="A14" s="8" t="s">
@@ -1519,26 +1534,26 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:A13"/>
+    <mergeCell ref="B6:B13"/>
+    <mergeCell ref="C6:C13"/>
+    <mergeCell ref="D6:D13"/>
+    <mergeCell ref="E6:E13"/>
+    <mergeCell ref="F6:F13"/>
+    <mergeCell ref="G6:G13"/>
+    <mergeCell ref="H6:H13"/>
+    <mergeCell ref="I6:I13"/>
+    <mergeCell ref="J6:J13"/>
+    <mergeCell ref="K6:K13"/>
+    <mergeCell ref="L6:L13"/>
+    <mergeCell ref="M6:M13"/>
+    <mergeCell ref="N6:N13"/>
     <mergeCell ref="O6:O13"/>
     <mergeCell ref="P6:P13"/>
     <mergeCell ref="Q6:Q13"/>
     <mergeCell ref="R6:R13"/>
     <mergeCell ref="S6:S13"/>
-    <mergeCell ref="J6:J13"/>
-    <mergeCell ref="K6:K13"/>
-    <mergeCell ref="L6:L13"/>
-    <mergeCell ref="M6:M13"/>
-    <mergeCell ref="N6:N13"/>
-    <mergeCell ref="E6:E13"/>
-    <mergeCell ref="F6:F13"/>
-    <mergeCell ref="G6:G13"/>
-    <mergeCell ref="H6:H13"/>
-    <mergeCell ref="I6:I13"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A6:A13"/>
-    <mergeCell ref="B6:B13"/>
-    <mergeCell ref="C6:C13"/>
-    <mergeCell ref="D6:D13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1547,23 +1562,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.625" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="5.75" customWidth="1"/>
     <col min="2" max="3" width="14.25" customWidth="1"/>
     <col min="4" max="4" width="11.375" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="17.125" customWidth="1"/>
+    <col min="6" max="6" width="21.25" customWidth="1"/>
     <col min="7" max="7" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="29"/>
@@ -1996,51 +2011,101 @@
       <c r="F21" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G21" s="30"/>
+      <c r="G21" s="30">
+        <v>3</v>
+      </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="29">
         <v>19</v>
       </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
+      <c r="B22" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="38">
+        <v>46230</v>
+      </c>
+      <c r="D22" s="30">
+        <v>31</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="30">
+        <v>5</v>
+      </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="29">
         <v>20</v>
       </c>
-      <c r="B23" s="30"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
+      <c r="B23" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="38">
+        <v>46231</v>
+      </c>
+      <c r="D23" s="30">
+        <v>31</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G23" s="30">
+        <v>4</v>
+      </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="29">
         <v>21</v>
       </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
+      <c r="B24" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="38">
+        <v>46231</v>
+      </c>
+      <c r="D24" s="30">
+        <v>31</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G24" s="30">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="29">
         <v>22</v>
       </c>
-      <c r="B25" s="30"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="30"/>
+      <c r="B25" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="38">
+        <v>46231</v>
+      </c>
+      <c r="D25" s="30">
+        <v>31</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G25" s="30">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="29">
@@ -2053,16 +2118,49 @@
       <c r="F26" s="30"/>
       <c r="G26" s="30"/>
     </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="29">
+        <v>24</v>
+      </c>
+      <c r="B27" s="30"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="29">
+        <v>25</v>
+      </c>
+      <c r="B28" s="30"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="29">
+        <v>26</v>
+      </c>
+      <c r="B29" s="30"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+    </row>
     <row r="31" spans="1:7" ht="15">
       <c r="A31" s="13" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="46" t="s">
+      <c r="A32" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B32" s="46"/>
+      <c r="B32" s="54"/>
       <c r="C32" s="29" t="s">
         <v>62</v>
       </c>
@@ -2080,10 +2178,10 @@
       </c>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="52" t="s">
+      <c r="A33" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="52"/>
+      <c r="B33" s="55"/>
       <c r="C33" s="32">
         <v>16</v>
       </c>
@@ -2096,15 +2194,15 @@
         <v>1</v>
       </c>
       <c r="F33" s="35"/>
-      <c r="G33" s="54" t="s">
+      <c r="G33" s="41" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="51" t="s">
+      <c r="A34" s="53" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="51"/>
+      <c r="B34" s="53"/>
       <c r="C34" s="17">
         <v>8</v>
       </c>
@@ -2117,15 +2215,15 @@
         <v>9.4705882352941178</v>
       </c>
       <c r="F34" s="35"/>
-      <c r="G34" s="53" t="s">
+      <c r="G34" s="40" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="51" t="s">
+      <c r="A35" s="53" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="51"/>
+      <c r="B35" s="53"/>
       <c r="C35" s="17">
         <v>8</v>
       </c>
@@ -2138,15 +2236,15 @@
         <v>2.125</v>
       </c>
       <c r="F35" s="35"/>
-      <c r="G35" s="54" t="s">
+      <c r="G35" s="41" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="49" t="s">
+      <c r="A36" s="51" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="50"/>
+      <c r="B36" s="52"/>
       <c r="C36" s="17">
         <v>4</v>
       </c>
@@ -2159,15 +2257,15 @@
         <v>3.32258064516129</v>
       </c>
       <c r="F36" s="35"/>
-      <c r="G36" s="54" t="s">
+      <c r="G36" s="41" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="51" t="s">
+      <c r="A37" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="51"/>
+      <c r="B37" s="53"/>
       <c r="C37" s="17">
         <f>SUM($C33:$C36)</f>
         <v>36</v>
@@ -2181,15 +2279,15 @@
         <v>7.25</v>
       </c>
       <c r="F37" s="35"/>
-      <c r="G37" s="55" t="s">
+      <c r="G37" s="42" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="46" t="s">
+      <c r="A39" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B39" s="46"/>
+      <c r="B39" s="54"/>
       <c r="C39" s="29" t="s">
         <v>62</v>
       </c>
@@ -2207,29 +2305,31 @@
       </c>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="47" t="s">
+      <c r="A40" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B40" s="48"/>
+      <c r="B40" s="50"/>
       <c r="C40" s="14">
         <v>8</v>
       </c>
       <c r="D40" s="4">
         <f t="shared" ref="D40:D47" si="0">SUMIFS($G$4:$G$1002,$F$4:$F$1002,$A40,$E$4:$E$1002,"BauhallenUhr")</f>
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E40" s="34">
         <f t="shared" ref="E40:E48" si="1">IF($C40&lt;$D40, $C40/$D40*9+1, $D40/$C40*9+1)</f>
-        <v>8.1999999999999993</v>
+        <v>4.7894736842105257</v>
       </c>
       <c r="F40" s="34"/>
-      <c r="G40" s="4"/>
+      <c r="G40" s="56" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="47" t="s">
+      <c r="A41" s="49" t="s">
         <v>50</v>
       </c>
-      <c r="B41" s="48"/>
+      <c r="B41" s="50"/>
       <c r="C41" s="14">
         <v>8</v>
       </c>
@@ -2245,48 +2345,48 @@
       <c r="G41" s="4"/>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="47" t="s">
+      <c r="A42" s="49" t="s">
         <v>51</v>
       </c>
-      <c r="B42" s="48"/>
+      <c r="B42" s="50"/>
       <c r="C42" s="14">
         <v>8</v>
       </c>
       <c r="D42" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E42" s="34">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>1.5625</v>
       </c>
       <c r="F42" s="34"/>
       <c r="G42" s="4"/>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="47" t="s">
+      <c r="A43" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="48"/>
+      <c r="B43" s="50"/>
       <c r="C43" s="14">
         <v>40</v>
       </c>
       <c r="D43" s="4">
         <f t="shared" si="0"/>
-        <v>34.5</v>
+        <v>38.5</v>
       </c>
       <c r="E43" s="34">
         <f t="shared" si="1"/>
-        <v>8.7624999999999993</v>
+        <v>9.6624999999999996</v>
       </c>
       <c r="F43" s="33"/>
       <c r="G43" s="4"/>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="47" t="s">
+      <c r="A44" s="49" t="s">
         <v>52</v>
       </c>
-      <c r="B44" s="48"/>
+      <c r="B44" s="50"/>
       <c r="C44" s="14">
         <v>40</v>
       </c>
@@ -2302,10 +2402,10 @@
       <c r="G44" s="4"/>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="47" t="s">
+      <c r="A45" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="B45" s="48"/>
+      <c r="B45" s="50"/>
       <c r="C45" s="14">
         <v>20</v>
       </c>
@@ -2321,10 +2421,10 @@
       <c r="G45" s="4"/>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="47" t="s">
+      <c r="A46" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="B46" s="48"/>
+      <c r="B46" s="50"/>
       <c r="C46" s="14">
         <v>15</v>
       </c>
@@ -2340,10 +2440,10 @@
       <c r="G46" s="4"/>
     </row>
     <row r="47" spans="1:7">
-      <c r="A47" s="47" t="s">
+      <c r="A47" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="B47" s="48"/>
+      <c r="B47" s="50"/>
       <c r="C47" s="14">
         <v>15</v>
       </c>
@@ -2359,21 +2459,21 @@
       <c r="G47" s="4"/>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="47" t="s">
+      <c r="A48" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="B48" s="48"/>
+      <c r="B48" s="50"/>
       <c r="C48" s="14">
         <f>SUM($C40:$C47)</f>
         <v>154</v>
       </c>
       <c r="D48" s="4">
         <f>SUM(D40:D47)</f>
-        <v>44.5</v>
+        <v>58</v>
       </c>
       <c r="E48" s="34">
         <f t="shared" si="1"/>
-        <v>3.6006493506493507</v>
+        <v>4.3896103896103895</v>
       </c>
       <c r="F48" s="33"/>
       <c r="G48" s="4"/>
@@ -2390,13 +2490,28 @@
         <v>67</v>
       </c>
     </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="57" t="s">
+        <v>77</v>
+      </c>
+      <c r="B53" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="57"/>
+      <c r="B54" t="s">
+        <v>78</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A48:B48"/>
+  <mergeCells count="18">
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A40:B40"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="A1:C1"/>
@@ -2404,11 +2519,11 @@
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Optokoppler - Ergänzung begonnen.
</commit_message>
<xml_diff>
--- a/Bauhalle_Zeitplan_woechentlich.xlsx
+++ b/Bauhalle_Zeitplan_woechentlich.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hueppim\Documents\Github\BauhallenUhr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F10DA9-8EC2-45B0-99CC-8F1CA9DC77D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA2C353-4FCC-4F96-84B5-AF768FA96EB1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44385" yWindow="3855" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3855" windowWidth="21570" windowHeight="5385" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zeitplan wöchentlich" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="79">
   <si>
     <t>Bauhalle Zeitplan wöchentlich</t>
   </si>
@@ -681,6 +681,9 @@
     <xf numFmtId="0" fontId="10" fillId="12" borderId="2" xfId="8" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="2" xfId="10" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -696,12 +699,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -721,7 +718,10 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1003,11 +1003,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="21" customHeight="1">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
     </row>
     <row r="3" spans="1:19" ht="15">
       <c r="A3" s="3" t="s">
@@ -1151,194 +1151,194 @@
       </c>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="48" t="s">
+      <c r="B6" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="C6" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="45" t="s">
+      <c r="D6" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="45" t="s">
+      <c r="E6" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="45" t="s">
+      <c r="F6" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="46" t="s">
+      <c r="G6" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="45" t="s">
+      <c r="I6" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="45" t="s">
+      <c r="J6" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
-      <c r="N6" s="43"/>
-      <c r="O6" s="43"/>
-      <c r="P6" s="43"/>
-      <c r="Q6" s="43"/>
-      <c r="R6" s="43"/>
-      <c r="S6" s="44" t="s">
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="44"/>
+      <c r="O6" s="44"/>
+      <c r="P6" s="44"/>
+      <c r="Q6" s="44"/>
+      <c r="R6" s="44"/>
+      <c r="S6" s="45" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:19">
-      <c r="A7" s="43"/>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
-      <c r="I7" s="43"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
-      <c r="N7" s="43"/>
-      <c r="O7" s="43"/>
-      <c r="P7" s="43"/>
-      <c r="Q7" s="43"/>
-      <c r="R7" s="43"/>
-      <c r="S7" s="44"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
+      <c r="N7" s="44"/>
+      <c r="O7" s="44"/>
+      <c r="P7" s="44"/>
+      <c r="Q7" s="44"/>
+      <c r="R7" s="44"/>
+      <c r="S7" s="45"/>
     </row>
     <row r="8" spans="1:19">
-      <c r="A8" s="43"/>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="43"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="43"/>
-      <c r="N8" s="43"/>
-      <c r="O8" s="43"/>
-      <c r="P8" s="43"/>
-      <c r="Q8" s="43"/>
-      <c r="R8" s="43"/>
-      <c r="S8" s="44"/>
+      <c r="A8" s="44"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="44"/>
+      <c r="O8" s="44"/>
+      <c r="P8" s="44"/>
+      <c r="Q8" s="44"/>
+      <c r="R8" s="44"/>
+      <c r="S8" s="45"/>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="43"/>
-      <c r="B9" s="43"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="43"/>
-      <c r="I9" s="43"/>
-      <c r="J9" s="43"/>
-      <c r="K9" s="43"/>
-      <c r="L9" s="43"/>
-      <c r="M9" s="43"/>
-      <c r="N9" s="43"/>
-      <c r="O9" s="43"/>
-      <c r="P9" s="43"/>
-      <c r="Q9" s="43"/>
-      <c r="R9" s="43"/>
-      <c r="S9" s="44"/>
+      <c r="A9" s="44"/>
+      <c r="B9" s="44"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="44"/>
+      <c r="L9" s="44"/>
+      <c r="M9" s="44"/>
+      <c r="N9" s="44"/>
+      <c r="O9" s="44"/>
+      <c r="P9" s="44"/>
+      <c r="Q9" s="44"/>
+      <c r="R9" s="44"/>
+      <c r="S9" s="45"/>
     </row>
     <row r="10" spans="1:19">
-      <c r="A10" s="43"/>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43"/>
-      <c r="I10" s="43"/>
-      <c r="J10" s="43"/>
-      <c r="K10" s="43"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="43"/>
-      <c r="N10" s="43"/>
-      <c r="O10" s="43"/>
-      <c r="P10" s="43"/>
-      <c r="Q10" s="43"/>
-      <c r="R10" s="43"/>
-      <c r="S10" s="44"/>
+      <c r="A10" s="44"/>
+      <c r="B10" s="44"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="44"/>
+      <c r="M10" s="44"/>
+      <c r="N10" s="44"/>
+      <c r="O10" s="44"/>
+      <c r="P10" s="44"/>
+      <c r="Q10" s="44"/>
+      <c r="R10" s="44"/>
+      <c r="S10" s="45"/>
     </row>
     <row r="11" spans="1:19">
-      <c r="A11" s="43"/>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="43"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="43"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-      <c r="O11" s="43"/>
-      <c r="P11" s="43"/>
-      <c r="Q11" s="43"/>
-      <c r="R11" s="43"/>
-      <c r="S11" s="44"/>
+      <c r="A11" s="44"/>
+      <c r="B11" s="44"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="44"/>
+      <c r="M11" s="44"/>
+      <c r="N11" s="44"/>
+      <c r="O11" s="44"/>
+      <c r="P11" s="44"/>
+      <c r="Q11" s="44"/>
+      <c r="R11" s="44"/>
+      <c r="S11" s="45"/>
     </row>
     <row r="12" spans="1:19">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-      <c r="K12" s="43"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="43"/>
-      <c r="N12" s="43"/>
-      <c r="O12" s="43"/>
-      <c r="P12" s="43"/>
-      <c r="Q12" s="43"/>
-      <c r="R12" s="43"/>
-      <c r="S12" s="44"/>
+      <c r="A12" s="44"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="44"/>
+      <c r="M12" s="44"/>
+      <c r="N12" s="44"/>
+      <c r="O12" s="44"/>
+      <c r="P12" s="44"/>
+      <c r="Q12" s="44"/>
+      <c r="R12" s="44"/>
+      <c r="S12" s="45"/>
     </row>
     <row r="13" spans="1:19">
-      <c r="A13" s="43"/>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43"/>
-      <c r="K13" s="43"/>
-      <c r="L13" s="43"/>
-      <c r="M13" s="43"/>
-      <c r="N13" s="43"/>
-      <c r="O13" s="43"/>
-      <c r="P13" s="43"/>
-      <c r="Q13" s="43"/>
-      <c r="R13" s="43"/>
-      <c r="S13" s="44"/>
+      <c r="A13" s="44"/>
+      <c r="B13" s="44"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="45"/>
     </row>
     <row r="14" spans="1:19" ht="30" customHeight="1">
       <c r="A14" s="8" t="s">
@@ -1574,11 +1574,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" customHeight="1">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="48" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="29"/>
@@ -2111,12 +2111,24 @@
       <c r="A26" s="29">
         <v>23</v>
       </c>
-      <c r="B26" s="30"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
+      <c r="B26" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="38">
+        <v>46232</v>
+      </c>
+      <c r="D26" s="30">
+        <v>31</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G26" s="30">
+        <v>9</v>
+      </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="29">
@@ -2157,10 +2169,10 @@
       </c>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="54" t="s">
+      <c r="A32" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="B32" s="54"/>
+      <c r="B32" s="53"/>
       <c r="C32" s="29" t="s">
         <v>62</v>
       </c>
@@ -2178,10 +2190,10 @@
       </c>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="55" t="s">
+      <c r="A33" s="54" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="55"/>
+      <c r="B33" s="54"/>
       <c r="C33" s="32">
         <v>16</v>
       </c>
@@ -2199,10 +2211,10 @@
       </c>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="53" t="s">
+      <c r="A34" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="53"/>
+      <c r="B34" s="52"/>
       <c r="C34" s="17">
         <v>8</v>
       </c>
@@ -2220,10 +2232,10 @@
       </c>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="53" t="s">
+      <c r="A35" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="53"/>
+      <c r="B35" s="52"/>
       <c r="C35" s="17">
         <v>8</v>
       </c>
@@ -2241,10 +2253,10 @@
       </c>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="51" t="s">
+      <c r="A36" s="50" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="52"/>
+      <c r="B36" s="51"/>
       <c r="C36" s="17">
         <v>4</v>
       </c>
@@ -2262,10 +2274,10 @@
       </c>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="53" t="s">
+      <c r="A37" s="52" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="53"/>
+      <c r="B37" s="52"/>
       <c r="C37" s="17">
         <f>SUM($C33:$C36)</f>
         <v>36</v>
@@ -2284,10 +2296,10 @@
       </c>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="54" t="s">
+      <c r="A39" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="B39" s="54"/>
+      <c r="B39" s="53"/>
       <c r="C39" s="29" t="s">
         <v>62</v>
       </c>
@@ -2305,10 +2317,10 @@
       </c>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="49" t="s">
+      <c r="A40" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="B40" s="50"/>
+      <c r="B40" s="57"/>
       <c r="C40" s="14">
         <v>8</v>
       </c>
@@ -2321,15 +2333,15 @@
         <v>4.7894736842105257</v>
       </c>
       <c r="F40" s="34"/>
-      <c r="G40" s="56" t="s">
+      <c r="G40" s="43" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="49" t="s">
+      <c r="A41" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="B41" s="50"/>
+      <c r="B41" s="57"/>
       <c r="C41" s="14">
         <v>8</v>
       </c>
@@ -2345,10 +2357,10 @@
       <c r="G41" s="4"/>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="49" t="s">
+      <c r="A42" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="B42" s="50"/>
+      <c r="B42" s="57"/>
       <c r="C42" s="14">
         <v>8</v>
       </c>
@@ -2364,29 +2376,29 @@
       <c r="G42" s="4"/>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="49" t="s">
+      <c r="A43" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="50"/>
+      <c r="B43" s="57"/>
       <c r="C43" s="14">
         <v>40</v>
       </c>
       <c r="D43" s="4">
         <f t="shared" si="0"/>
-        <v>38.5</v>
+        <v>47.5</v>
       </c>
       <c r="E43" s="34">
         <f t="shared" si="1"/>
-        <v>9.6624999999999996</v>
+        <v>8.5789473684210513</v>
       </c>
       <c r="F43" s="33"/>
       <c r="G43" s="4"/>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="49" t="s">
+      <c r="A44" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="B44" s="50"/>
+      <c r="B44" s="57"/>
       <c r="C44" s="14">
         <v>40</v>
       </c>
@@ -2402,10 +2414,10 @@
       <c r="G44" s="4"/>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="49" t="s">
+      <c r="A45" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="B45" s="50"/>
+      <c r="B45" s="57"/>
       <c r="C45" s="14">
         <v>20</v>
       </c>
@@ -2421,10 +2433,10 @@
       <c r="G45" s="4"/>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="49" t="s">
+      <c r="A46" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="B46" s="50"/>
+      <c r="B46" s="57"/>
       <c r="C46" s="14">
         <v>15</v>
       </c>
@@ -2440,10 +2452,10 @@
       <c r="G46" s="4"/>
     </row>
     <row r="47" spans="1:7">
-      <c r="A47" s="49" t="s">
+      <c r="A47" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="B47" s="50"/>
+      <c r="B47" s="57"/>
       <c r="C47" s="14">
         <v>15</v>
       </c>
@@ -2459,21 +2471,21 @@
       <c r="G47" s="4"/>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="49" t="s">
+      <c r="A48" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="B48" s="50"/>
+      <c r="B48" s="57"/>
       <c r="C48" s="14">
         <f>SUM($C40:$C47)</f>
         <v>154</v>
       </c>
       <c r="D48" s="4">
         <f>SUM(D40:D47)</f>
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E48" s="34">
         <f t="shared" si="1"/>
-        <v>4.3896103896103895</v>
+        <v>4.9155844155844157</v>
       </c>
       <c r="F48" s="33"/>
       <c r="G48" s="4"/>
@@ -2491,7 +2503,7 @@
       </c>
     </row>
     <row r="53" spans="1:2">
-      <c r="A53" s="57" t="s">
+      <c r="A53" s="55" t="s">
         <v>77</v>
       </c>
       <c r="B53" t="s">
@@ -2499,7 +2511,7 @@
       </c>
     </row>
     <row r="54" spans="1:2">
-      <c r="A54" s="57"/>
+      <c r="A54" s="55"/>
       <c r="B54" t="s">
         <v>78</v>
       </c>
@@ -2512,6 +2524,11 @@
     <mergeCell ref="A42:B42"/>
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="A1:C1"/>
@@ -2519,11 +2536,6 @@
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A48:B48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Kommentare bei Zeitplanung hinzugefügt.
</commit_message>
<xml_diff>
--- a/Bauhalle_Zeitplan_woechentlich.xlsx
+++ b/Bauhalle_Zeitplan_woechentlich.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hueppim\Documents\Github\BauhallenUhr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{273078D7-81C6-4A55-B521-E7213D56BF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8211F95-B6F5-45CA-A1F4-3E244E69D91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44385" yWindow="3855" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="81">
   <si>
     <t>Bauhalle Zeitplan wöchentlich</t>
   </si>
@@ -276,13 +276,22 @@
   </si>
   <si>
     <t>Dazu habe ich vergessen, die Bauteilauswahl bei Elektronische Bauteile einzuschreiben.</t>
+  </si>
+  <si>
+    <t>**</t>
+  </si>
+  <si>
+    <t>Nicht schlecht eingeschätzt, Abweichung von 25%. Muss im Hinblick auf IPA verbessert werden.
+Dazu darf die Zeit fürs Schema nicht 40h betragen, sondern eher 10h oder max. 15h.
+Beim Schema sollte ich mehr mit vorgefertigten Komponenten und Symbolen/ Footprints arbeiten, dadurch spare ich eine Menge Zeit.
+Ich sollte für die IPA dann auch meinen "Perfektionismus" ablegen.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,6 +385,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -460,7 +476,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -610,6 +626,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -624,7 +682,7 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -695,46 +753,95 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="4" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="4" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="2" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="5" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="7" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="10" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Excel Built-in 20% - Accent1" xfId="7" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
@@ -1014,11 +1121,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -1162,194 +1269,194 @@
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="55" t="s">
+      <c r="D6" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="55" t="s">
+      <c r="E6" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="55" t="s">
+      <c r="F6" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="56" t="s">
+      <c r="G6" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="55" t="s">
+      <c r="H6" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="55" t="s">
+      <c r="I6" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="55" t="s">
+      <c r="J6" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="53"/>
-      <c r="L6" s="53"/>
-      <c r="M6" s="53"/>
-      <c r="N6" s="53"/>
-      <c r="O6" s="53"/>
-      <c r="P6" s="53"/>
-      <c r="Q6" s="53"/>
-      <c r="R6" s="53"/>
-      <c r="S6" s="57" t="s">
+      <c r="K6" s="52"/>
+      <c r="L6" s="52"/>
+      <c r="M6" s="52"/>
+      <c r="N6" s="52"/>
+      <c r="O6" s="52"/>
+      <c r="P6" s="52"/>
+      <c r="Q6" s="52"/>
+      <c r="R6" s="52"/>
+      <c r="S6" s="53" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" s="53"/>
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="53"/>
-      <c r="K7" s="53"/>
-      <c r="L7" s="53"/>
-      <c r="M7" s="53"/>
-      <c r="N7" s="53"/>
-      <c r="O7" s="53"/>
-      <c r="P7" s="53"/>
-      <c r="Q7" s="53"/>
-      <c r="R7" s="53"/>
-      <c r="S7" s="57"/>
+      <c r="A7" s="52"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="52"/>
+      <c r="F7" s="52"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="52"/>
+      <c r="L7" s="52"/>
+      <c r="M7" s="52"/>
+      <c r="N7" s="52"/>
+      <c r="O7" s="52"/>
+      <c r="P7" s="52"/>
+      <c r="Q7" s="52"/>
+      <c r="R7" s="52"/>
+      <c r="S7" s="53"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" s="53"/>
-      <c r="B8" s="53"/>
-      <c r="C8" s="53"/>
-      <c r="D8" s="53"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="53"/>
-      <c r="G8" s="53"/>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="53"/>
-      <c r="K8" s="53"/>
-      <c r="L8" s="53"/>
-      <c r="M8" s="53"/>
-      <c r="N8" s="53"/>
-      <c r="O8" s="53"/>
-      <c r="P8" s="53"/>
-      <c r="Q8" s="53"/>
-      <c r="R8" s="53"/>
-      <c r="S8" s="57"/>
+      <c r="A8" s="52"/>
+      <c r="B8" s="52"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
+      <c r="G8" s="52"/>
+      <c r="H8" s="52"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="52"/>
+      <c r="K8" s="52"/>
+      <c r="L8" s="52"/>
+      <c r="M8" s="52"/>
+      <c r="N8" s="52"/>
+      <c r="O8" s="52"/>
+      <c r="P8" s="52"/>
+      <c r="Q8" s="52"/>
+      <c r="R8" s="52"/>
+      <c r="S8" s="53"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A9" s="53"/>
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="53"/>
-      <c r="E9" s="53"/>
-      <c r="F9" s="53"/>
-      <c r="G9" s="53"/>
-      <c r="H9" s="53"/>
-      <c r="I9" s="53"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
-      <c r="M9" s="53"/>
-      <c r="N9" s="53"/>
-      <c r="O9" s="53"/>
-      <c r="P9" s="53"/>
-      <c r="Q9" s="53"/>
-      <c r="R9" s="53"/>
-      <c r="S9" s="57"/>
+      <c r="A9" s="52"/>
+      <c r="B9" s="52"/>
+      <c r="C9" s="52"/>
+      <c r="D9" s="52"/>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="52"/>
+      <c r="K9" s="52"/>
+      <c r="L9" s="52"/>
+      <c r="M9" s="52"/>
+      <c r="N9" s="52"/>
+      <c r="O9" s="52"/>
+      <c r="P9" s="52"/>
+      <c r="Q9" s="52"/>
+      <c r="R9" s="52"/>
+      <c r="S9" s="53"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10" s="53"/>
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="53"/>
-      <c r="F10" s="53"/>
-      <c r="G10" s="53"/>
-      <c r="H10" s="53"/>
-      <c r="I10" s="53"/>
-      <c r="J10" s="53"/>
-      <c r="K10" s="53"/>
-      <c r="L10" s="53"/>
-      <c r="M10" s="53"/>
-      <c r="N10" s="53"/>
-      <c r="O10" s="53"/>
-      <c r="P10" s="53"/>
-      <c r="Q10" s="53"/>
-      <c r="R10" s="53"/>
-      <c r="S10" s="57"/>
+      <c r="A10" s="52"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="52"/>
+      <c r="D10" s="52"/>
+      <c r="E10" s="52"/>
+      <c r="F10" s="52"/>
+      <c r="G10" s="52"/>
+      <c r="H10" s="52"/>
+      <c r="I10" s="52"/>
+      <c r="J10" s="52"/>
+      <c r="K10" s="52"/>
+      <c r="L10" s="52"/>
+      <c r="M10" s="52"/>
+      <c r="N10" s="52"/>
+      <c r="O10" s="52"/>
+      <c r="P10" s="52"/>
+      <c r="Q10" s="52"/>
+      <c r="R10" s="52"/>
+      <c r="S10" s="53"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" s="53"/>
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
-      <c r="D11" s="53"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="53"/>
-      <c r="G11" s="53"/>
-      <c r="H11" s="53"/>
-      <c r="I11" s="53"/>
-      <c r="J11" s="53"/>
-      <c r="K11" s="53"/>
-      <c r="L11" s="53"/>
-      <c r="M11" s="53"/>
-      <c r="N11" s="53"/>
-      <c r="O11" s="53"/>
-      <c r="P11" s="53"/>
-      <c r="Q11" s="53"/>
-      <c r="R11" s="53"/>
-      <c r="S11" s="57"/>
+      <c r="A11" s="52"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="52"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="52"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="52"/>
+      <c r="M11" s="52"/>
+      <c r="N11" s="52"/>
+      <c r="O11" s="52"/>
+      <c r="P11" s="52"/>
+      <c r="Q11" s="52"/>
+      <c r="R11" s="52"/>
+      <c r="S11" s="53"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
-      <c r="D12" s="53"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="53"/>
-      <c r="G12" s="53"/>
-      <c r="H12" s="53"/>
-      <c r="I12" s="53"/>
-      <c r="J12" s="53"/>
-      <c r="K12" s="53"/>
-      <c r="L12" s="53"/>
-      <c r="M12" s="53"/>
-      <c r="N12" s="53"/>
-      <c r="O12" s="53"/>
-      <c r="P12" s="53"/>
-      <c r="Q12" s="53"/>
-      <c r="R12" s="53"/>
-      <c r="S12" s="57"/>
+      <c r="A12" s="52"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="52"/>
+      <c r="J12" s="52"/>
+      <c r="K12" s="52"/>
+      <c r="L12" s="52"/>
+      <c r="M12" s="52"/>
+      <c r="N12" s="52"/>
+      <c r="O12" s="52"/>
+      <c r="P12" s="52"/>
+      <c r="Q12" s="52"/>
+      <c r="R12" s="52"/>
+      <c r="S12" s="53"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13" s="53"/>
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
-      <c r="D13" s="53"/>
-      <c r="E13" s="53"/>
-      <c r="F13" s="53"/>
-      <c r="G13" s="53"/>
-      <c r="H13" s="53"/>
-      <c r="I13" s="53"/>
-      <c r="J13" s="53"/>
-      <c r="K13" s="53"/>
-      <c r="L13" s="53"/>
-      <c r="M13" s="53"/>
-      <c r="N13" s="53"/>
-      <c r="O13" s="53"/>
-      <c r="P13" s="53"/>
-      <c r="Q13" s="53"/>
-      <c r="R13" s="53"/>
-      <c r="S13" s="57"/>
+      <c r="A13" s="52"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="52"/>
+      <c r="D13" s="52"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="52"/>
+      <c r="J13" s="52"/>
+      <c r="K13" s="52"/>
+      <c r="L13" s="52"/>
+      <c r="M13" s="52"/>
+      <c r="N13" s="52"/>
+      <c r="O13" s="52"/>
+      <c r="P13" s="52"/>
+      <c r="Q13" s="52"/>
+      <c r="R13" s="52"/>
+      <c r="S13" s="53"/>
     </row>
     <row r="14" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
@@ -1545,26 +1652,26 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:A13"/>
+    <mergeCell ref="B6:B13"/>
+    <mergeCell ref="C6:C13"/>
+    <mergeCell ref="D6:D13"/>
+    <mergeCell ref="E6:E13"/>
+    <mergeCell ref="F6:F13"/>
+    <mergeCell ref="G6:G13"/>
+    <mergeCell ref="H6:H13"/>
+    <mergeCell ref="I6:I13"/>
+    <mergeCell ref="J6:J13"/>
+    <mergeCell ref="K6:K13"/>
+    <mergeCell ref="L6:L13"/>
+    <mergeCell ref="M6:M13"/>
+    <mergeCell ref="N6:N13"/>
     <mergeCell ref="O6:O13"/>
     <mergeCell ref="P6:P13"/>
     <mergeCell ref="Q6:Q13"/>
     <mergeCell ref="R6:R13"/>
     <mergeCell ref="S6:S13"/>
-    <mergeCell ref="J6:J13"/>
-    <mergeCell ref="K6:K13"/>
-    <mergeCell ref="L6:L13"/>
-    <mergeCell ref="M6:M13"/>
-    <mergeCell ref="N6:N13"/>
-    <mergeCell ref="E6:E13"/>
-    <mergeCell ref="F6:F13"/>
-    <mergeCell ref="G6:G13"/>
-    <mergeCell ref="H6:H13"/>
-    <mergeCell ref="I6:I13"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A6:A13"/>
-    <mergeCell ref="B6:B13"/>
-    <mergeCell ref="C6:C13"/>
-    <mergeCell ref="D6:D13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1573,7 +1680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
@@ -1585,11 +1692,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="29"/>
@@ -2161,7 +2268,7 @@
         <v>31</v>
       </c>
       <c r="G27" s="30">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -2192,10 +2299,10 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="45" t="s">
+      <c r="A32" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="B32" s="45"/>
+      <c r="B32" s="48"/>
       <c r="C32" s="29" t="s">
         <v>62</v>
       </c>
@@ -2213,15 +2320,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="52" t="s">
+      <c r="A33" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="52"/>
+      <c r="B33" s="49"/>
       <c r="C33" s="32">
         <v>16</v>
       </c>
       <c r="D33" s="28">
-        <f>SUMIFS($G$4:$G$1002,$F$4:$F$1002,$A33,$E$4:$E$1002,"Thermostat")</f>
+        <f>SUMIFS($G$4:$G$1003,$F$4:$F$1003,$A33,$E$4:$E$1003,"Thermostat")</f>
         <v>0</v>
       </c>
       <c r="E33" s="33">
@@ -2234,15 +2341,15 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="50" t="s">
+      <c r="A34" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="50"/>
+      <c r="B34" s="46"/>
       <c r="C34" s="17">
         <v>8</v>
       </c>
       <c r="D34" s="4">
-        <f>SUMIFS($G$4:$G$1002,$F$4:$F$1002,$A34,$E$4:$E$1002,"Thermostat")</f>
+        <f>SUMIFS($G$4:$G$1003,$F$4:$F$1003,$A34,$E$4:$E$1003,"Thermostat")</f>
         <v>8.5</v>
       </c>
       <c r="E34" s="34">
@@ -2255,15 +2362,15 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="50" t="s">
+      <c r="A35" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="50"/>
+      <c r="B35" s="46"/>
       <c r="C35" s="17">
         <v>8</v>
       </c>
       <c r="D35" s="4">
-        <f>SUMIFS($G$4:$G$1002,$F$4:$F$1002,$A35,$E$4:$E$1002,"Thermostat")</f>
+        <f>SUMIFS($G$4:$G$1003,$F$4:$F$1003,$A35,$E$4:$E$1003,"Thermostat")</f>
         <v>1</v>
       </c>
       <c r="E35" s="34">
@@ -2276,15 +2383,15 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="48" t="s">
+      <c r="A36" s="44" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="49"/>
+      <c r="B36" s="45"/>
       <c r="C36" s="17">
         <v>4</v>
       </c>
       <c r="D36" s="4">
-        <f>SUMIFS($G$4:$G$1002,$F$4:$F$1002,$A36,$E$4:$E$1002,"Thermostat")</f>
+        <f>SUMIFS($G$4:$G$1003,$F$4:$F$1003,$A36,$E$4:$E$1003,"Thermostat")</f>
         <v>15.5</v>
       </c>
       <c r="E36" s="34">
@@ -2297,10 +2404,10 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="50" t="s">
+      <c r="A37" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="50"/>
+      <c r="B37" s="46"/>
       <c r="C37" s="17">
         <f>SUM($C33:$C36)</f>
         <v>36</v>
@@ -2319,10 +2426,10 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="45" t="s">
+      <c r="A39" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="B39" s="45"/>
+      <c r="B39" s="48"/>
       <c r="C39" s="29" t="s">
         <v>62</v>
       </c>
@@ -2340,31 +2447,31 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="46" t="s">
+      <c r="A40" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="B40" s="47"/>
+      <c r="B40" s="51"/>
       <c r="C40" s="14">
         <v>8</v>
       </c>
       <c r="D40" s="4">
-        <f t="shared" ref="D40:D47" si="0">SUMIFS($G$4:$G$1002,$F$4:$F$1002,$A40,$E$4:$E$1002,"BauhallenUhr")</f>
+        <f t="shared" ref="D40:D47" si="0">SUMIFS($G$4:$G$1003,$F$4:$F$1003,$A40,$E$4:$E$1003,"BauhallenUhr")</f>
         <v>19</v>
       </c>
       <c r="E40" s="34">
         <f t="shared" ref="E40:E48" si="1">IF($C40&lt;$D40, $C40/$D40*9+1, $D40/$C40*9+1)</f>
         <v>4.7894736842105257</v>
       </c>
-      <c r="F40" s="34"/>
+      <c r="F40" s="35"/>
       <c r="G40" s="43" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="46" t="s">
+      <c r="A41" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="B41" s="47"/>
+      <c r="B41" s="51"/>
       <c r="C41" s="14">
         <v>8</v>
       </c>
@@ -2380,10 +2487,10 @@
       <c r="G41" s="4"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="46" t="s">
+      <c r="A42" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="B42" s="47"/>
+      <c r="B42" s="51"/>
       <c r="C42" s="14">
         <v>8</v>
       </c>
@@ -2396,32 +2503,36 @@
         <v>1.5625</v>
       </c>
       <c r="F42" s="34"/>
-      <c r="G42" s="4"/>
+      <c r="G42" s="43" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="46" t="s">
+      <c r="A43" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="47"/>
+      <c r="B43" s="51"/>
       <c r="C43" s="14">
         <v>40</v>
       </c>
       <c r="D43" s="4">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>49.5</v>
       </c>
       <c r="E43" s="34">
         <f t="shared" si="1"/>
-        <v>8.3469387755102034</v>
-      </c>
-      <c r="F43" s="33"/>
-      <c r="G43" s="4"/>
+        <v>8.2727272727272734</v>
+      </c>
+      <c r="F43" s="35"/>
+      <c r="G43" s="57" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="46" t="s">
+      <c r="A44" s="50" t="s">
         <v>52</v>
       </c>
-      <c r="B44" s="47"/>
+      <c r="B44" s="51"/>
       <c r="C44" s="14">
         <v>40</v>
       </c>
@@ -2437,10 +2548,10 @@
       <c r="G44" s="4"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="46" t="s">
+      <c r="A45" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="B45" s="47"/>
+      <c r="B45" s="51"/>
       <c r="C45" s="14">
         <v>20</v>
       </c>
@@ -2456,10 +2567,10 @@
       <c r="G45" s="4"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="46" t="s">
+      <c r="A46" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="B46" s="47"/>
+      <c r="B46" s="51"/>
       <c r="C46" s="14">
         <v>15</v>
       </c>
@@ -2475,10 +2586,10 @@
       <c r="G46" s="4"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="46" t="s">
+      <c r="A47" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="B47" s="47"/>
+      <c r="B47" s="51"/>
       <c r="C47" s="14">
         <v>15</v>
       </c>
@@ -2494,61 +2605,128 @@
       <c r="G47" s="4"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="46" t="s">
+      <c r="A48" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="B48" s="47"/>
+      <c r="B48" s="51"/>
       <c r="C48" s="14">
         <f>SUM($C40:$C47)</f>
         <v>154</v>
       </c>
       <c r="D48" s="4">
         <f>SUM(D40:D47)</f>
-        <v>68.5</v>
+        <v>69</v>
       </c>
       <c r="E48" s="34">
         <f t="shared" si="1"/>
-        <v>5.0032467532467537</v>
+        <v>5.0324675324675319</v>
       </c>
       <c r="F48" s="33"/>
       <c r="G48" s="4"/>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="19"/>
       <c r="B50" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="36"/>
       <c r="B51" s="4" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="44" t="s">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" s="74" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="43" t="s">
         <v>77</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B54" s="58" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="44"/>
-      <c r="B54" t="s">
+      <c r="C54" s="58"/>
+      <c r="D54" s="58"/>
+      <c r="E54" s="58"/>
+      <c r="F54" s="58"/>
+      <c r="G54" s="58"/>
+      <c r="H54" s="58"/>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="B55" s="59" t="s">
         <v>78</v>
       </c>
+      <c r="C55" s="60"/>
+      <c r="D55" s="60"/>
+      <c r="E55" s="60"/>
+      <c r="F55" s="60"/>
+      <c r="G55" s="60"/>
+      <c r="H55" s="61"/>
+    </row>
+    <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="71" t="s">
+        <v>77</v>
+      </c>
+      <c r="B57" s="62" t="s">
+        <v>80</v>
+      </c>
+      <c r="C57" s="63"/>
+      <c r="D57" s="63"/>
+      <c r="E57" s="63"/>
+      <c r="F57" s="63"/>
+      <c r="G57" s="63"/>
+      <c r="H57" s="63"/>
+      <c r="I57" s="63"/>
+      <c r="J57" s="64"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="72"/>
+      <c r="B58" s="65"/>
+      <c r="C58" s="66"/>
+      <c r="D58" s="66"/>
+      <c r="E58" s="66"/>
+      <c r="F58" s="66"/>
+      <c r="G58" s="66"/>
+      <c r="H58" s="66"/>
+      <c r="I58" s="66"/>
+      <c r="J58" s="67"/>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="72"/>
+      <c r="B59" s="65"/>
+      <c r="C59" s="66"/>
+      <c r="D59" s="66"/>
+      <c r="E59" s="66"/>
+      <c r="F59" s="66"/>
+      <c r="G59" s="66"/>
+      <c r="H59" s="66"/>
+      <c r="I59" s="66"/>
+      <c r="J59" s="67"/>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" s="73"/>
+      <c r="B60" s="68"/>
+      <c r="C60" s="69"/>
+      <c r="D60" s="69"/>
+      <c r="E60" s="69"/>
+      <c r="F60" s="69"/>
+      <c r="G60" s="69"/>
+      <c r="H60" s="69"/>
+      <c r="I60" s="69"/>
+      <c r="J60" s="70"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A53:A54"/>
+  <mergeCells count="21">
+    <mergeCell ref="A57:A60"/>
+    <mergeCell ref="B57:J60"/>
+    <mergeCell ref="B54:H54"/>
+    <mergeCell ref="B55:H55"/>
     <mergeCell ref="A39:B39"/>
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="A42:B42"/>
@@ -2559,6 +2737,13 @@
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Zwischenstand gespeichtert um an anderem PC zu arbeiten.
</commit_message>
<xml_diff>
--- a/Bauhalle_Zeitplan_woechentlich.xlsx
+++ b/Bauhalle_Zeitplan_woechentlich.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8211F95-B6F5-45CA-A1F4-3E244E69D91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44385" yWindow="3855" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6165" yWindow="3225" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zeitplan wöchentlich" sheetId="1" r:id="rId1"/>
@@ -753,6 +753,67 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="2" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="5" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="7" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="10" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -763,85 +824,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="4" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="2" xfId="10" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="5" xfId="10" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="7" xfId="10" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="10" xfId="10" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Excel Built-in 20% - Accent1" xfId="7" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
@@ -1121,11 +1121,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -1269,194 +1269,194 @@
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="70" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="54" t="s">
+      <c r="D6" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="54" t="s">
+      <c r="E6" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="54" t="s">
+      <c r="F6" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="55" t="s">
+      <c r="G6" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="54" t="s">
+      <c r="H6" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="54" t="s">
+      <c r="I6" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="54" t="s">
+      <c r="J6" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="52"/>
-      <c r="L6" s="52"/>
-      <c r="M6" s="52"/>
-      <c r="N6" s="52"/>
-      <c r="O6" s="52"/>
-      <c r="P6" s="52"/>
-      <c r="Q6" s="52"/>
-      <c r="R6" s="52"/>
-      <c r="S6" s="53" t="s">
+      <c r="K6" s="70"/>
+      <c r="L6" s="70"/>
+      <c r="M6" s="70"/>
+      <c r="N6" s="70"/>
+      <c r="O6" s="70"/>
+      <c r="P6" s="70"/>
+      <c r="Q6" s="70"/>
+      <c r="R6" s="70"/>
+      <c r="S6" s="74" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" s="52"/>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
-      <c r="G7" s="52"/>
-      <c r="H7" s="52"/>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="52"/>
-      <c r="L7" s="52"/>
-      <c r="M7" s="52"/>
-      <c r="N7" s="52"/>
-      <c r="O7" s="52"/>
-      <c r="P7" s="52"/>
-      <c r="Q7" s="52"/>
-      <c r="R7" s="52"/>
-      <c r="S7" s="53"/>
+      <c r="A7" s="70"/>
+      <c r="B7" s="70"/>
+      <c r="C7" s="70"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="70"/>
+      <c r="H7" s="70"/>
+      <c r="I7" s="70"/>
+      <c r="J7" s="70"/>
+      <c r="K7" s="70"/>
+      <c r="L7" s="70"/>
+      <c r="M7" s="70"/>
+      <c r="N7" s="70"/>
+      <c r="O7" s="70"/>
+      <c r="P7" s="70"/>
+      <c r="Q7" s="70"/>
+      <c r="R7" s="70"/>
+      <c r="S7" s="74"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" s="52"/>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="52"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="52"/>
-      <c r="L8" s="52"/>
-      <c r="M8" s="52"/>
-      <c r="N8" s="52"/>
-      <c r="O8" s="52"/>
-      <c r="P8" s="52"/>
-      <c r="Q8" s="52"/>
-      <c r="R8" s="52"/>
-      <c r="S8" s="53"/>
+      <c r="A8" s="70"/>
+      <c r="B8" s="70"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="70"/>
+      <c r="E8" s="70"/>
+      <c r="F8" s="70"/>
+      <c r="G8" s="70"/>
+      <c r="H8" s="70"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="70"/>
+      <c r="K8" s="70"/>
+      <c r="L8" s="70"/>
+      <c r="M8" s="70"/>
+      <c r="N8" s="70"/>
+      <c r="O8" s="70"/>
+      <c r="P8" s="70"/>
+      <c r="Q8" s="70"/>
+      <c r="R8" s="70"/>
+      <c r="S8" s="74"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A9" s="52"/>
-      <c r="B9" s="52"/>
-      <c r="C9" s="52"/>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
-      <c r="G9" s="52"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="52"/>
-      <c r="J9" s="52"/>
-      <c r="K9" s="52"/>
-      <c r="L9" s="52"/>
-      <c r="M9" s="52"/>
-      <c r="N9" s="52"/>
-      <c r="O9" s="52"/>
-      <c r="P9" s="52"/>
-      <c r="Q9" s="52"/>
-      <c r="R9" s="52"/>
-      <c r="S9" s="53"/>
+      <c r="A9" s="70"/>
+      <c r="B9" s="70"/>
+      <c r="C9" s="70"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="70"/>
+      <c r="G9" s="70"/>
+      <c r="H9" s="70"/>
+      <c r="I9" s="70"/>
+      <c r="J9" s="70"/>
+      <c r="K9" s="70"/>
+      <c r="L9" s="70"/>
+      <c r="M9" s="70"/>
+      <c r="N9" s="70"/>
+      <c r="O9" s="70"/>
+      <c r="P9" s="70"/>
+      <c r="Q9" s="70"/>
+      <c r="R9" s="70"/>
+      <c r="S9" s="74"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
-      <c r="B10" s="52"/>
-      <c r="C10" s="52"/>
-      <c r="D10" s="52"/>
-      <c r="E10" s="52"/>
-      <c r="F10" s="52"/>
-      <c r="G10" s="52"/>
-      <c r="H10" s="52"/>
-      <c r="I10" s="52"/>
-      <c r="J10" s="52"/>
-      <c r="K10" s="52"/>
-      <c r="L10" s="52"/>
-      <c r="M10" s="52"/>
-      <c r="N10" s="52"/>
-      <c r="O10" s="52"/>
-      <c r="P10" s="52"/>
-      <c r="Q10" s="52"/>
-      <c r="R10" s="52"/>
-      <c r="S10" s="53"/>
+      <c r="A10" s="70"/>
+      <c r="B10" s="70"/>
+      <c r="C10" s="70"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="70"/>
+      <c r="H10" s="70"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="70"/>
+      <c r="K10" s="70"/>
+      <c r="L10" s="70"/>
+      <c r="M10" s="70"/>
+      <c r="N10" s="70"/>
+      <c r="O10" s="70"/>
+      <c r="P10" s="70"/>
+      <c r="Q10" s="70"/>
+      <c r="R10" s="70"/>
+      <c r="S10" s="74"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
-      <c r="B11" s="52"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
-      <c r="I11" s="52"/>
-      <c r="J11" s="52"/>
-      <c r="K11" s="52"/>
-      <c r="L11" s="52"/>
-      <c r="M11" s="52"/>
-      <c r="N11" s="52"/>
-      <c r="O11" s="52"/>
-      <c r="P11" s="52"/>
-      <c r="Q11" s="52"/>
-      <c r="R11" s="52"/>
-      <c r="S11" s="53"/>
+      <c r="A11" s="70"/>
+      <c r="B11" s="70"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="70"/>
+      <c r="G11" s="70"/>
+      <c r="H11" s="70"/>
+      <c r="I11" s="70"/>
+      <c r="J11" s="70"/>
+      <c r="K11" s="70"/>
+      <c r="L11" s="70"/>
+      <c r="M11" s="70"/>
+      <c r="N11" s="70"/>
+      <c r="O11" s="70"/>
+      <c r="P11" s="70"/>
+      <c r="Q11" s="70"/>
+      <c r="R11" s="70"/>
+      <c r="S11" s="74"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="52"/>
-      <c r="B12" s="52"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-      <c r="I12" s="52"/>
-      <c r="J12" s="52"/>
-      <c r="K12" s="52"/>
-      <c r="L12" s="52"/>
-      <c r="M12" s="52"/>
-      <c r="N12" s="52"/>
-      <c r="O12" s="52"/>
-      <c r="P12" s="52"/>
-      <c r="Q12" s="52"/>
-      <c r="R12" s="52"/>
-      <c r="S12" s="53"/>
+      <c r="A12" s="70"/>
+      <c r="B12" s="70"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="70"/>
+      <c r="G12" s="70"/>
+      <c r="H12" s="70"/>
+      <c r="I12" s="70"/>
+      <c r="J12" s="70"/>
+      <c r="K12" s="70"/>
+      <c r="L12" s="70"/>
+      <c r="M12" s="70"/>
+      <c r="N12" s="70"/>
+      <c r="O12" s="70"/>
+      <c r="P12" s="70"/>
+      <c r="Q12" s="70"/>
+      <c r="R12" s="70"/>
+      <c r="S12" s="74"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13" s="52"/>
-      <c r="B13" s="52"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="52"/>
-      <c r="F13" s="52"/>
-      <c r="G13" s="52"/>
-      <c r="H13" s="52"/>
-      <c r="I13" s="52"/>
-      <c r="J13" s="52"/>
-      <c r="K13" s="52"/>
-      <c r="L13" s="52"/>
-      <c r="M13" s="52"/>
-      <c r="N13" s="52"/>
-      <c r="O13" s="52"/>
-      <c r="P13" s="52"/>
-      <c r="Q13" s="52"/>
-      <c r="R13" s="52"/>
-      <c r="S13" s="53"/>
+      <c r="A13" s="70"/>
+      <c r="B13" s="70"/>
+      <c r="C13" s="70"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="70"/>
+      <c r="H13" s="70"/>
+      <c r="I13" s="70"/>
+      <c r="J13" s="70"/>
+      <c r="K13" s="70"/>
+      <c r="L13" s="70"/>
+      <c r="M13" s="70"/>
+      <c r="N13" s="70"/>
+      <c r="O13" s="70"/>
+      <c r="P13" s="70"/>
+      <c r="Q13" s="70"/>
+      <c r="R13" s="70"/>
+      <c r="S13" s="74"/>
     </row>
     <row r="14" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
@@ -1652,26 +1652,26 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="O6:O13"/>
+    <mergeCell ref="P6:P13"/>
+    <mergeCell ref="Q6:Q13"/>
+    <mergeCell ref="R6:R13"/>
+    <mergeCell ref="S6:S13"/>
+    <mergeCell ref="J6:J13"/>
+    <mergeCell ref="K6:K13"/>
+    <mergeCell ref="L6:L13"/>
+    <mergeCell ref="M6:M13"/>
+    <mergeCell ref="N6:N13"/>
+    <mergeCell ref="E6:E13"/>
+    <mergeCell ref="F6:F13"/>
+    <mergeCell ref="G6:G13"/>
+    <mergeCell ref="H6:H13"/>
+    <mergeCell ref="I6:I13"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A6:A13"/>
     <mergeCell ref="B6:B13"/>
     <mergeCell ref="C6:C13"/>
     <mergeCell ref="D6:D13"/>
-    <mergeCell ref="E6:E13"/>
-    <mergeCell ref="F6:F13"/>
-    <mergeCell ref="G6:G13"/>
-    <mergeCell ref="H6:H13"/>
-    <mergeCell ref="I6:I13"/>
-    <mergeCell ref="J6:J13"/>
-    <mergeCell ref="K6:K13"/>
-    <mergeCell ref="L6:L13"/>
-    <mergeCell ref="M6:M13"/>
-    <mergeCell ref="N6:N13"/>
-    <mergeCell ref="O6:O13"/>
-    <mergeCell ref="P6:P13"/>
-    <mergeCell ref="Q6:Q13"/>
-    <mergeCell ref="R6:R13"/>
-    <mergeCell ref="S6:S13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1692,11 +1692,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="29"/>
@@ -2299,10 +2299,10 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="48" t="s">
+      <c r="A32" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="62"/>
       <c r="C32" s="29" t="s">
         <v>62</v>
       </c>
@@ -2320,10 +2320,10 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="49" t="s">
+      <c r="A33" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="49"/>
+      <c r="B33" s="69"/>
       <c r="C33" s="32">
         <v>16</v>
       </c>
@@ -2341,10 +2341,10 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="46" t="s">
+      <c r="A34" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="46"/>
+      <c r="B34" s="67"/>
       <c r="C34" s="17">
         <v>8</v>
       </c>
@@ -2362,10 +2362,10 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="46" t="s">
+      <c r="A35" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="46"/>
+      <c r="B35" s="67"/>
       <c r="C35" s="17">
         <v>8</v>
       </c>
@@ -2383,10 +2383,10 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="44" t="s">
+      <c r="A36" s="65" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="45"/>
+      <c r="B36" s="66"/>
       <c r="C36" s="17">
         <v>4</v>
       </c>
@@ -2404,10 +2404,10 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="46" t="s">
+      <c r="A37" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="46"/>
+      <c r="B37" s="67"/>
       <c r="C37" s="17">
         <f>SUM($C33:$C36)</f>
         <v>36</v>
@@ -2426,10 +2426,10 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="48" t="s">
+      <c r="A39" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="B39" s="48"/>
+      <c r="B39" s="62"/>
       <c r="C39" s="29" t="s">
         <v>62</v>
       </c>
@@ -2447,10 +2447,10 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="50" t="s">
+      <c r="A40" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="B40" s="51"/>
+      <c r="B40" s="64"/>
       <c r="C40" s="14">
         <v>8</v>
       </c>
@@ -2468,10 +2468,10 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="50" t="s">
+      <c r="A41" s="63" t="s">
         <v>50</v>
       </c>
-      <c r="B41" s="51"/>
+      <c r="B41" s="64"/>
       <c r="C41" s="14">
         <v>8</v>
       </c>
@@ -2487,10 +2487,10 @@
       <c r="G41" s="4"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="50" t="s">
+      <c r="A42" s="63" t="s">
         <v>51</v>
       </c>
-      <c r="B42" s="51"/>
+      <c r="B42" s="64"/>
       <c r="C42" s="14">
         <v>8</v>
       </c>
@@ -2508,10 +2508,10 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="50" t="s">
+      <c r="A43" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="51"/>
+      <c r="B43" s="64"/>
       <c r="C43" s="14">
         <v>40</v>
       </c>
@@ -2524,15 +2524,15 @@
         <v>8.2727272727272734</v>
       </c>
       <c r="F43" s="35"/>
-      <c r="G43" s="57" t="s">
+      <c r="G43" s="44" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="50" t="s">
+      <c r="A44" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="B44" s="51"/>
+      <c r="B44" s="64"/>
       <c r="C44" s="14">
         <v>40</v>
       </c>
@@ -2548,10 +2548,10 @@
       <c r="G44" s="4"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="50" t="s">
+      <c r="A45" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B45" s="51"/>
+      <c r="B45" s="64"/>
       <c r="C45" s="14">
         <v>20</v>
       </c>
@@ -2567,10 +2567,10 @@
       <c r="G45" s="4"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="50" t="s">
+      <c r="A46" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="B46" s="51"/>
+      <c r="B46" s="64"/>
       <c r="C46" s="14">
         <v>15</v>
       </c>
@@ -2586,10 +2586,10 @@
       <c r="G46" s="4"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="50" t="s">
+      <c r="A47" s="63" t="s">
         <v>35</v>
       </c>
-      <c r="B47" s="51"/>
+      <c r="B47" s="64"/>
       <c r="C47" s="14">
         <v>15</v>
       </c>
@@ -2605,10 +2605,10 @@
       <c r="G47" s="4"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="50" t="s">
+      <c r="A48" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="B48" s="51"/>
+      <c r="B48" s="64"/>
       <c r="C48" s="14">
         <f>SUM($C40:$C47)</f>
         <v>154</v>
@@ -2637,7 +2637,7 @@
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A53" s="74" t="s">
+      <c r="A53" s="45" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2670,59 +2670,66 @@
       <c r="H55" s="61"/>
     </row>
     <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="71" t="s">
+      <c r="A57" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="B57" s="62" t="s">
+      <c r="B57" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="C57" s="63"/>
-      <c r="D57" s="63"/>
-      <c r="E57" s="63"/>
-      <c r="F57" s="63"/>
-      <c r="G57" s="63"/>
-      <c r="H57" s="63"/>
-      <c r="I57" s="63"/>
-      <c r="J57" s="64"/>
+      <c r="C57" s="50"/>
+      <c r="D57" s="50"/>
+      <c r="E57" s="50"/>
+      <c r="F57" s="50"/>
+      <c r="G57" s="50"/>
+      <c r="H57" s="50"/>
+      <c r="I57" s="50"/>
+      <c r="J57" s="51"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A58" s="72"/>
-      <c r="B58" s="65"/>
-      <c r="C58" s="66"/>
-      <c r="D58" s="66"/>
-      <c r="E58" s="66"/>
-      <c r="F58" s="66"/>
-      <c r="G58" s="66"/>
-      <c r="H58" s="66"/>
-      <c r="I58" s="66"/>
-      <c r="J58" s="67"/>
+      <c r="A58" s="47"/>
+      <c r="B58" s="52"/>
+      <c r="C58" s="53"/>
+      <c r="D58" s="53"/>
+      <c r="E58" s="53"/>
+      <c r="F58" s="53"/>
+      <c r="G58" s="53"/>
+      <c r="H58" s="53"/>
+      <c r="I58" s="53"/>
+      <c r="J58" s="54"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="72"/>
-      <c r="B59" s="65"/>
-      <c r="C59" s="66"/>
-      <c r="D59" s="66"/>
-      <c r="E59" s="66"/>
-      <c r="F59" s="66"/>
-      <c r="G59" s="66"/>
-      <c r="H59" s="66"/>
-      <c r="I59" s="66"/>
-      <c r="J59" s="67"/>
+      <c r="A59" s="47"/>
+      <c r="B59" s="52"/>
+      <c r="C59" s="53"/>
+      <c r="D59" s="53"/>
+      <c r="E59" s="53"/>
+      <c r="F59" s="53"/>
+      <c r="G59" s="53"/>
+      <c r="H59" s="53"/>
+      <c r="I59" s="53"/>
+      <c r="J59" s="54"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" s="73"/>
-      <c r="B60" s="68"/>
-      <c r="C60" s="69"/>
-      <c r="D60" s="69"/>
-      <c r="E60" s="69"/>
-      <c r="F60" s="69"/>
-      <c r="G60" s="69"/>
-      <c r="H60" s="69"/>
-      <c r="I60" s="69"/>
-      <c r="J60" s="70"/>
+      <c r="A60" s="48"/>
+      <c r="B60" s="55"/>
+      <c r="C60" s="56"/>
+      <c r="D60" s="56"/>
+      <c r="E60" s="56"/>
+      <c r="F60" s="56"/>
+      <c r="G60" s="56"/>
+      <c r="H60" s="56"/>
+      <c r="I60" s="56"/>
+      <c r="J60" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="A57:A60"/>
     <mergeCell ref="B57:J60"/>
     <mergeCell ref="B54:H54"/>
@@ -2737,13 +2744,6 @@
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>